<commit_message>
Record resilient Cerberus Telegram fallback
</commit_message>
<xml_diff>
--- a/kurultai-feature-status.xlsx
+++ b/kurultai-feature-status.xlsx
@@ -5328,7 +5328,7 @@
       </c>
       <c r="K81" s="10" t="inlineStr">
         <is>
-          <t>Direct and Hermes one-shot passed.</t>
+          <t>Direct, Hermes, and Kublai fallback one-shots passed; the local endpoint is managed by launchd.</t>
         </is>
       </c>
     </row>
@@ -21407,7 +21407,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>2026-06-23T01:50:08.067Z</t>
+          <t>2026-06-23T02:01:45.728Z</t>
         </is>
       </c>
     </row>

</xml_diff>